<commit_message>
Add rich text formatting support and update docs
Introduced rich text formatting support for product descriptions, allowing bold and color styles to be preserved from Excel to JSON and back. Updated README and added documentation guides. Refreshed Excel and JSON templates to reflect new formatting features. Removed obsolete color variants from JSON templates and batch files.
</commit_message>
<xml_diff>
--- a/order_generation/PO_excel/17-A1KN-KJGW-1.xlsx
+++ b/order_generation/PO_excel/17-A1KN-KJGW-1.xlsx
@@ -800,7 +800,7 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>2025年10月09日</t>
+          <t>2025年10月22日</t>
         </is>
       </c>
       <c r="H4" s="16" t="n"/>
@@ -996,7 +996,7 @@
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>2025年10月16日</t>
+          <t>2025年10月29日</t>
         </is>
       </c>
       <c r="C14" s="25" t="n"/>

</xml_diff>